<commit_message>
Add Demo logo file
</commit_message>
<xml_diff>
--- a/demo/data.xlsx
+++ b/demo/data.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -31,6 +34,15 @@
     <t xml:space="preserve">Mentor</t>
   </si>
   <si>
+    <t xml:space="preserve">website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID232</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sammy joe</t>
   </si>
   <si>
@@ -40,13 +52,28 @@
     <t xml:space="preserve">Mathew</t>
   </si>
   <si>
+    <t xml:space="preserve">https://shahil-sk.github.io</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/mnt/godown/PROJECTS/21_Active/certy/demo/logo.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID233</t>
+  </si>
+  <si>
     <t xml:space="preserve">John smith</t>
   </si>
   <si>
+    <t xml:space="preserve">ID234</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zoe</t>
   </si>
   <si>
     <t xml:space="preserve">jack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID235</t>
   </si>
   <si>
     <t xml:space="preserve">Ronald</t>
@@ -62,11 +89,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -82,6 +110,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -126,8 +161,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -254,65 +297,119 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.47"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" display="https://shahil-sk.github.io"/>
+    <hyperlink ref="E3" r:id="rId2" display="https://shahil-sk.github.io"/>
+    <hyperlink ref="E4" r:id="rId3" display="https://shahil-sk.github.io"/>
+    <hyperlink ref="E5" r:id="rId4" display="https://shahil-sk.github.io"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>